<commit_message>
fix: sync-cards.bat 윈도우 배치 파일 CRLF 및 CMD 구문 오류 수정
</commit_message>
<xml_diff>
--- a/src/data/roguelike-cards.xlsx
+++ b/src/data/roguelike-cards.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tak\Projects\dps-fire-mage\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3AA7B61-70F3-4DCF-934C-AFF0019BDA17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D217724-52E5-46F6-9786-825AEC26AB9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-36260" yWindow="1630" windowWidth="30020" windowHeight="17950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -383,9 +383,6 @@
     <t>🌀</t>
   </si>
   <si>
-    <t>화염구 시전 완료 시 4초간 시전 속도가 &lt;b&gt;+15%&lt;/b&gt; 가속됩니다 (최대 5중첩).</t>
-  </si>
-  <si>
     <t>haste_stack</t>
   </si>
   <si>
@@ -1059,6 +1056,10 @@
   </si>
   <si>
     <t>몬스터 처치 및 보스 격파 시 드롭되는 골드 획득량 증가</t>
+  </si>
+  <si>
+    <t>화염구 시전 완료 시 4초간 시전 속도가 &lt;b&gt;+15%&lt;/b&gt; 가속됩니다 (최대 2중첩).</t>
+    <phoneticPr fontId="8" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1749,7 +1750,7 @@
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>35</v>
+        <v>260</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1759,22 +1760,22 @@
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P5" s="2"/>
     </row>
     <row r="6" spans="1:16" ht="24" customHeight="1">
       <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="15" t="s">
         <v>39</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>40</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>20</v>
@@ -1783,7 +1784,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -1793,31 +1794,31 @@
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="P6" s="2"/>
     </row>
     <row r="7" spans="1:16" ht="24" customHeight="1">
       <c r="A7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>45</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F7" s="3">
         <v>5</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1833,25 +1834,25 @@
     </row>
     <row r="8" spans="1:16" ht="24" customHeight="1">
       <c r="A8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="D8" s="17" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F8" s="3">
         <v>5</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1867,25 +1868,25 @@
     </row>
     <row r="9" spans="1:16" ht="24" customHeight="1">
       <c r="A9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F9" s="3">
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -1893,37 +1894,37 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="P9" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="24" customHeight="1">
       <c r="A10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F10" s="3">
         <v>2</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -1931,35 +1932,35 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P10" s="2"/>
     </row>
     <row r="11" spans="1:16" ht="24" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="D11" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F11" s="3">
         <v>1</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -1967,20 +1968,20 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P11" s="2"/>
     </row>
     <row r="12" spans="1:16" ht="24" customHeight="1">
       <c r="A12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>70</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>24</v>
@@ -1989,13 +1990,13 @@
         <v>19</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F12" s="3">
         <v>4</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
@@ -2005,31 +2006,31 @@
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="P12" s="2"/>
     </row>
     <row r="13" spans="1:16" ht="24" customHeight="1">
       <c r="A13" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F13" s="3">
         <v>3</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
@@ -2037,37 +2038,37 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="P13" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="24" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>83</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F14" s="3">
         <v>1</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -2075,35 +2076,35 @@
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="P14" s="2"/>
     </row>
     <row r="15" spans="1:16" ht="24" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="D15" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F15" s="3">
         <v>1</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -2111,35 +2112,35 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="P15" s="2"/>
     </row>
     <row r="16" spans="1:16" ht="24" customHeight="1">
       <c r="A16" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>92</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>93</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F16" s="3">
         <v>3</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
@@ -2153,25 +2154,25 @@
     </row>
     <row r="17" spans="1:16" ht="24" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>97</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>98</v>
       </c>
       <c r="D17" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F17" s="3">
         <v>2</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -2181,33 +2182,33 @@
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="P17" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="P17" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="24" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>104</v>
-      </c>
       <c r="D18" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F18" s="3">
         <v>1</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -2215,35 +2216,35 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P18" s="2"/>
     </row>
     <row r="19" spans="1:16" ht="24" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>109</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>110</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>19</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F19" s="3">
         <v>1</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -2251,20 +2252,20 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" s="2"/>
     </row>
     <row r="20" spans="1:16" ht="24" customHeight="1">
       <c r="A20" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>28</v>
@@ -2273,13 +2274,13 @@
         <v>19</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F20" s="3">
         <v>1</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
@@ -2288,32 +2289,32 @@
       <c r="L20" s="3"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" s="2"/>
     </row>
     <row r="21" spans="1:16" ht="24" customHeight="1">
       <c r="A21" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>118</v>
-      </c>
       <c r="C21" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D21" s="16" t="s">
         <v>29</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F21" s="3">
         <v>1</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
@@ -2322,20 +2323,20 @@
       <c r="L21" s="3"/>
       <c r="M21" s="2"/>
       <c r="N21" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" s="2"/>
     </row>
     <row r="22" spans="1:16" ht="24" customHeight="1">
       <c r="A22" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="C22" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="16" t="s">
         <v>29</v>
@@ -2347,7 +2348,7 @@
         <v>1</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
@@ -2356,32 +2357,32 @@
       <c r="L22" s="3"/>
       <c r="M22" s="2"/>
       <c r="N22" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O22" s="2"/>
       <c r="P22" s="2"/>
     </row>
     <row r="23" spans="1:16" ht="24" customHeight="1">
       <c r="A23" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F23" s="3">
         <v>1</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
@@ -2390,7 +2391,7 @@
       <c r="L23" s="3"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" s="2"/>
@@ -2431,12 +2432,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21">
       <c r="A1" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="26" customHeight="1">
       <c r="A3" s="14" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -2444,7 +2445,7 @@
     </row>
     <row r="4" spans="1:4" ht="20" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -2452,16 +2453,16 @@
     </row>
     <row r="5" spans="1:4" ht="24" customHeight="1">
       <c r="A5" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>134</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="22" customHeight="1">
@@ -2469,13 +2470,13 @@
         <v>19</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D6" s="8" t="s">
         <v>137</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="22" customHeight="1">
@@ -2483,46 +2484,46 @@
         <v>29</v>
       </c>
       <c r="B7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="11" t="s">
         <v>140</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="22" customHeight="1">
       <c r="A8" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>144</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="22" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="11" t="s">
         <v>147</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="26" customHeight="1">
       <c r="A12" s="14" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -2530,7 +2531,7 @@
     </row>
     <row r="13" spans="1:4" ht="20" customHeight="1">
       <c r="A13" s="12" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2538,16 +2539,16 @@
     </row>
     <row r="14" spans="1:4" ht="24" customHeight="1">
       <c r="A14" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="5" t="s">
-        <v>133</v>
-      </c>
       <c r="C14" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="22" customHeight="1">
@@ -2555,165 +2556,165 @@
         <v>20</v>
       </c>
       <c r="B15" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="D15" s="8" t="s">
         <v>154</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="22" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B16" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C16" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="D16" s="11" t="s">
         <v>157</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="22" customHeight="1">
       <c r="A17" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="D17" s="8" t="s">
         <v>161</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="22" customHeight="1">
       <c r="A18" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>163</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="D18" s="11" t="s">
         <v>165</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="22" customHeight="1">
       <c r="A19" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="C19" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="D19" s="8" t="s">
         <v>169</v>
-      </c>
-      <c r="D19" s="8" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="26" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
     </row>
     <row r="23" spans="1:4" ht="20" customHeight="1">
       <c r="A23" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
     </row>
     <row r="24" spans="1:4" ht="24" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>173</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="22" customHeight="1">
       <c r="A25" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="B25" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="C25" s="8" t="s">
         <v>176</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="22" customHeight="1">
       <c r="A26" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="C26" s="11" t="s">
         <v>178</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="22" customHeight="1">
       <c r="A27" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B27" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>180</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="22" customHeight="1">
       <c r="A28" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C28" s="11" t="s">
         <v>182</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="22" customHeight="1">
       <c r="A29" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="B29" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>185</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="22" customHeight="1">
       <c r="A30" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B30" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C30" s="11" t="s">
         <v>187</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="26" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
@@ -2721,7 +2722,7 @@
     </row>
     <row r="34" spans="1:4" ht="20" customHeight="1">
       <c r="A34" s="12" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
@@ -2729,105 +2730,105 @@
     </row>
     <row r="35" spans="1:4" ht="24" customHeight="1">
       <c r="A35" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>192</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="22" customHeight="1">
       <c r="A36" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="D36" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="22" customHeight="1">
       <c r="A37" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B37" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="C37" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="D37" s="11" t="s">
         <v>198</v>
-      </c>
-      <c r="D37" s="11" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="22" customHeight="1">
       <c r="A38" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B38" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="D38" s="8" t="s">
         <v>201</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="22" customHeight="1">
       <c r="A39" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B39" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="C39" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="C39" s="11" t="s">
+      <c r="D39" s="11" t="s">
         <v>204</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="22" customHeight="1">
       <c r="A40" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B40" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="D40" s="8" t="s">
         <v>207</v>
-      </c>
-      <c r="D40" s="8" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="22" customHeight="1">
       <c r="A41" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>209</v>
       </c>
-      <c r="B41" s="10" t="s">
+      <c r="C41" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="C41" s="11" t="s">
+      <c r="D41" s="11" t="s">
         <v>211</v>
-      </c>
-      <c r="D41" s="11" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="26" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
@@ -2835,7 +2836,7 @@
     </row>
     <row r="45" spans="1:4" ht="20" customHeight="1">
       <c r="A45" s="12" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
@@ -2843,16 +2844,16 @@
     </row>
     <row r="46" spans="1:4" ht="24" customHeight="1">
       <c r="A46" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B46" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="C46" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="22" customHeight="1">
@@ -2860,172 +2861,172 @@
         <v>31</v>
       </c>
       <c r="B47" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="D47" s="8" t="s">
         <v>220</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>221</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="22" customHeight="1">
       <c r="A48" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B48" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="C48" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="D48" s="11" t="s">
         <v>223</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="22" customHeight="1">
       <c r="A49" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B49" s="7" t="s">
+        <v>224</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="C49" s="8" t="s">
-        <v>226</v>
-      </c>
       <c r="D49" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="50" spans="1:4" ht="22" customHeight="1">
       <c r="A50" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>226</v>
+      </c>
+      <c r="C50" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="D50" s="11" t="s">
         <v>57</v>
-      </c>
-      <c r="B50" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="C50" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="22" customHeight="1">
       <c r="A51" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B51" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C51" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="C51" s="8" t="s">
-        <v>230</v>
-      </c>
       <c r="D51" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="22" customHeight="1">
       <c r="A52" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>230</v>
+      </c>
+      <c r="C52" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="C52" s="11" t="s">
-        <v>232</v>
-      </c>
       <c r="D52" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="22" customHeight="1">
       <c r="A53" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B53" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="C53" s="8" t="s">
         <v>233</v>
       </c>
-      <c r="C53" s="8" t="s">
-        <v>234</v>
-      </c>
       <c r="D53" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="22" customHeight="1">
       <c r="A54" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="D54" s="11" t="s">
         <v>79</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="C54" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="D54" s="11" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="22" customHeight="1">
       <c r="A55" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B55" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C55" s="8" t="s">
         <v>237</v>
       </c>
-      <c r="C55" s="8" t="s">
-        <v>238</v>
-      </c>
       <c r="D55" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="22" customHeight="1">
       <c r="A56" s="9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B56" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="C56" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="C56" s="11" t="s">
-        <v>240</v>
-      </c>
       <c r="D56" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="22" customHeight="1">
       <c r="A57" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="D57" s="8" t="s">
         <v>100</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="C57" s="8" t="s">
-        <v>242</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="22" customHeight="1">
       <c r="A58" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D58" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="26" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B61" s="13"/>
       <c r="C61" s="13"/>
@@ -3033,7 +3034,7 @@
     </row>
     <row r="62" spans="1:4" ht="20" customHeight="1">
       <c r="A62" s="12" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B62" s="13"/>
       <c r="C62" s="13"/>
@@ -3041,16 +3042,16 @@
     </row>
     <row r="63" spans="1:4" ht="24" customHeight="1">
       <c r="A63" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="B63" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="B63" s="5" t="s">
+      <c r="C63" s="5" t="s">
         <v>247</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="D63" s="5" t="s">
         <v>248</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="22" customHeight="1">
@@ -3058,13 +3059,13 @@
         <v>7</v>
       </c>
       <c r="B64" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C64" s="8" t="s">
         <v>250</v>
       </c>
-      <c r="C64" s="8" t="s">
+      <c r="D64" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="22" customHeight="1">
@@ -3072,13 +3073,13 @@
         <v>8</v>
       </c>
       <c r="B65" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="C65" s="11" t="s">
         <v>253</v>
       </c>
-      <c r="C65" s="11" t="s">
+      <c r="D65" s="11" t="s">
         <v>254</v>
-      </c>
-      <c r="D65" s="11" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="22" customHeight="1">
@@ -3086,13 +3087,13 @@
         <v>9</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D66" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="22" customHeight="1">
@@ -3100,13 +3101,13 @@
         <v>10</v>
       </c>
       <c r="B67" s="10" t="s">
+        <v>256</v>
+      </c>
+      <c r="C67" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="D67" s="11" t="s">
         <v>257</v>
-      </c>
-      <c r="C67" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="D67" s="11" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="68" spans="1:4" ht="22" customHeight="1">
@@ -3114,13 +3115,13 @@
         <v>11</v>
       </c>
       <c r="B68" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="D68" s="8" t="s">
         <v>259</v>
-      </c>
-      <c r="C68" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>